<commit_message>
Update test files and order templates
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/日常文件/execl模板下单/3.3V/KEC清关订单模板 (7).xlsx
+++ b/日常文件/execl模板下单/3.3V/KEC清关订单模板 (7).xlsx
@@ -276,7 +276,7 @@
     <t>Sale Platform URL</t>
   </si>
   <si>
-    <t>CACNTH998</t>
+    <t>KEC-TESTGX</t>
   </si>
   <si>
     <t>TESTBACK20221312334</t>
@@ -947,19 +947,13 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="等线"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -1445,137 +1439,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1589,9 +1583,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -2239,7 +2230,7 @@
       </c>
     </row>
     <row r="2" customFormat="1" ht="13" customHeight="1" spans="1:81">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>82</v>
       </c>
       <c r="C2" t="s">
@@ -2308,7 +2299,7 @@
       <c r="AG2">
         <v>21000</v>
       </c>
-      <c r="AH2" s="10" t="s">
+      <c r="AH2" s="9" t="s">
         <v>98</v>
       </c>
       <c r="AI2" t="s">
@@ -2374,7 +2365,7 @@
       <c r="BU2" t="s">
         <v>101</v>
       </c>
-      <c r="BV2" s="10" t="s">
+      <c r="BV2" s="9" t="s">
         <v>105</v>
       </c>
       <c r="BW2">

</xml_diff>